<commit_message>
update  files for FAIR instructions
</commit_message>
<xml_diff>
--- a/FAIR_instructions_with_parsed_columns.xlsx
+++ b/FAIR_instructions_with_parsed_columns.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:T5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,47 +476,57 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Recommended file formats</t>
+          <t>1-Suggested file formats for each data type</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Relevant tools and software</t>
+          <t>2-Tools for converting data to the suggested file formats</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Recommended dataset structure or standard</t>
+          <t>3-Suggested standard structure to organize the dataset</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Dataset organization details</t>
+          <t>4-Tools for organizing the dataset in the suggested structure</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Metadata and documentation files to include</t>
+          <t>5-Metadata and information that should be provided with the data</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Tools for metadata preparation and validation</t>
+          <t>6-Suggested standard structure and file format for metadata</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>De-identification and privacy considerations</t>
+          <t>7-Tools for preparing metadata in the suggested structure and file format</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Recommended repositories</t>
+          <t>8-Suggested de-identification approach</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Recommended data licenses</t>
+          <t>9-Tools to implement the suggested de-identification approach</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>10-Suggested repositories for sharing the dataset</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>11-Suggested license for sharing the dataset</t>
         </is>
       </c>
     </row>
@@ -564,24 +574,28 @@
 - If yes, data sharing consent: All research participants will be consented for broad data sharing.
 - Data to be collected: Demographic, clinical, and MRI, 1 H fMRS and fMRI imaging data will be acquired from 110 affected youth and 110 matched healthy controls (described in detail in sections C.3 and C.4 of this application). All data will be deidentified prior to receipt by the repository, but the information needed to generate a global unique identifier for the NIMH Data Archive (NDA) will be collected for each subject.
 Based on these inputs, provide clear, practical, and user-friendly FAIR data guidance organized under the following sections:
-1. Recommended file formats
-Explain which file format(s) should be used for this type of data and why they are appropriate for FAIR sharing and reuse.
-2. Relevant tools and software
-List tools, software, or platforms that can help prepare, convert, validate, organize, document, or share this type of data.
-3. Recommended dataset structure or standard
-State the dataset structure, schema, or community standard that should be followed, if one exists.
-4. Dataset organization details
-Provide detailed guidance on how the dataset should be organized, including folder structure, file naming conventions, table organization, metadata arrangement, versioning considerations, and any other important technical details.
-5. Metadata and documentation files to include
-List the metadata files, README files, data dictionaries, codebooks, protocols, or other documentation that should accompany the dataset.
-6. Tools for metadata preparation and validation
-Suggest tools that can help create, validate, manage, or standardize metadata for this dataset.
-7. De-identification and privacy considerations
-State whether de-identification is required. Explain what should be done based on the subject type, the data modality, and whether the study involves human participants. If consent language affects sharing, explain that clearly.
-8. Recommended repositories
-Suggest appropriate repositories for sharing the data, prioritizing repositories recommended, required, or commonly accepted by the funding source and data type.
-9. Recommended data licenses
-Recommend appropriate data license(s), prioritizing those expected, suggested, or required by the funding source. If restrictions apply because of human subjects or consent limitations, explain that clearly.
+1- Suggested file formats for each data type
+Identify the recommended file format or formats for each data type in the dataset. Briefly explain why these formats are appropriate for FAIR sharing, reuse, interoperability, and long-term preservation.
+2- Tools for converting data to the suggested file formats
+List tools, software, or workflows that can be used to convert raw or source data into the recommended file formats.
+3- Suggested standard structure to organize the dataset
+State the recommended dataset structure, schema, specification, or community standard that should be used to organize the dataset, if one exists.
+4- Tools for organizing the dataset in the suggested structure
+List tools, software, templates, or platforms that can help organize the dataset according to the recommended structure or standard.
+5- Metadata and information that should be provided with the data
+Describe the metadata, documentation, contextual information, data dictionaries, codebooks, README files, protocols, and any other supporting information that should accompany the dataset.
+6- Suggested standard structure and file format for metadata
+State the recommended structure, schema, standard, and file format that should be used for metadata and documentation files included with the dataset.
+7-Tools for preparing metadata in the suggested structure and file format
+List tools, software, validators, templates, or platforms that can help create, manage, standardize, or validate metadata in the recommended structure and format.
+8- Suggested de-identification approach
+State whether de-identification is required. Explain the recommended de-identification or privacy-preserving approach based on the subject type, data modality, sensitivity of the data, and whether human participants are involved. If consent language affects sharing, explain that clearly.
+9- Tools to implement the suggested de-identification approach
+List tools, software, workflows, or methods that can help implement the recommended de-identification or privacy protection approach.
+10-Suggested repositories for sharing the dataset
+Recommend appropriate repositories for sharing the dataset, prioritizing repositories required, recommended, or commonly accepted by the funding source, subject type, and data modality.
+11- Suggested license for sharing the dataset
+Recommend an appropriate data license or licensing approach, prioritizing what is expected, suggested, or required by the funding source. If restrictions apply because of human subjects, controlled access, or consent limitations, explain that clearly.
 Instructions for your response:
 - Make the guidance practical, concise, and easy for researchers to follow.
 - Tailor all recommendations to the combination of funding source, human-subject status, consent language, and data modality.
@@ -592,76 +606,100 @@
 Return your answer in valid JSON format only.
 Use exactly this JSON structure:
 {
-  "Recommended file formats": "",
-  "Relevant tools and software": "",
-  "Recommended dataset structure or standard": "",
-  "Dataset organization details": "",
-  "Metadata and documentation files to include": "",
-  "Tools for metadata preparation and validation": "",
-  "De-identification and privacy considerations": "",
-  "Recommended repositories": "",
-  "Recommended data licenses": ""
+  "1-Suggested file formats for each data type": "",
+  "2-Tools for converting data to the suggested file formats": "",
+  "3-Suggested standard structure to organize the dataset": "",
+  "4-Tools for organizing the dataset in the suggested structure": "",
+  "5-Metadata and information that should be provided with the data": "",
+  "6-Suggested standard structure and file format for metadata": "",
+  "7-Tools for preparing metadata in the suggested structure and file format": "",
+  "8-Suggested de-identification approach": "",
+  "9-Tools to implement the suggested de-identification approach": "",
+  "10-Suggested repositories for sharing the dataset": "",
+  "11-Suggested license for sharing the dataset": ""
 }</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>{
-  "Recommended file formats": "For imaging data (MRI, 1H fMRS, fMRI), use NIfTI (.nii or .nii.gz) for volumetric data and BIDS-compliant formats for associated metadata (e.g., .json sidecars). For raw scanner data, DICOM (.dcm) may be retained but should be converted to NIfTI for sharing. For tabular data (demographics, clinical), use non-proprietary formats such as CSV (.csv) or TSV (.tsv). Documentation and metadata should be provided in plain text (.txt), Markdown (.md), or PDF (.pdf) formats. These formats are open, widely supported, and facilitate interoperability and reuse.",
-  "Relevant tools and software": "Use dcm2niix for DICOM to NIfTI conversion; BIDS Validator for checking dataset compliance; MRIQC and fMRIPrep for quality control and preprocessing; PyBIDS for programmatic BIDS data handling; spreadsheet software (e.g., Excel, LibreOffice) for tabular data (export as CSV/TSV); and Git or similar version control for tracking changes. For documentation, use text editors or Markdown tools.",
-  "Recommended dataset structure or standard": "Follow the Brain Imaging Data Structure (BIDS) standard for organizing and describing MRI, fMRI, and fMRS data. For clinical and demographic data, use BIDS 'participants.tsv' and associated data dictionaries. BIDS is widely accepted in neuroimaging and required by many repositories, including the NIMH Data Archive (NDA).",
-  "Dataset organization details": "Organize data in a BIDS-compliant folder structure: a root directory with subfolders for each subject (e.g., sub-&lt;NDA_GUID&gt;), session folders if applicable, and modality-specific folders (anat, func, fmap, mrs, etc.). Use standardized BIDS file naming conventions (e.g., sub-&lt;NDA_GUID&gt;_ses-01_task-rest_bold.nii.gz). Store tabular data (demographics, clinical) in 'participants.tsv' and additional .tsv files as needed, with accompanying data dictionaries. Include a top-level README, dataset_description.json, and CHANGES file for versioning. Use consistent versioning for dataset updates and document changes in the CHANGES file.",
-  "Metadata and documentation files to include": "Include a README file describing the dataset, a dataset_description.json (per BIDS), participants.tsv (with data dictionary), and modality-specific .json sidecar files for imaging data. Provide a data dictionary/codebook for all tabular data, protocols for data collection and processing, and a CHANGES file for version history. If using NDA, include NDA-specific metadata files as required.",
-  "Tools for metadata preparation and validation": "Use the BIDS Validator (web or command-line) to check dataset and metadata compliance. The NDA Data Dictionary Tool can help prepare NDA-compliant metadata. For general metadata, tools like DataLad or CEDAR Workbench can assist with metadata management. Use spreadsheet software for data dictionaries, ensuring export to open formats.",
-  "De-identification and privacy considerations": "De-identification is required for all human subjects data. Remove all direct identifiers from imaging and tabular data. For imaging, use tools like pydeface or mri_deface to remove facial features from structural scans. Ensure no PHI remains in DICOM headers or tabular files. Collect and use the NDA Global Unique Identifier (GUID) for each subject to enable linkage without direct identifiers. Since participants are consented for broad data sharing, data can be shared in accordance with NIH and NDA policies, but always confirm that consent language aligns with intended sharing scope.",
-  "Recommended repositories": "Deposit all data in the NIMH Data Archive (NDA), as required for NIMH-funded human subjects research. NDA supports BIDS and provides infrastructure for secure, compliant sharing of deidentified human neuroimaging and associated data. Optionally, consider secondary sharing in OpenNeuro for broader community access, provided all NDA and consent requirements are met.",
-  "Recommended data licenses": "For NDA, data are shared under NDA's Data Use Certification, which governs access and reuse. If sharing in additional repositories (e.g., OpenNeuro), use the Creative Commons CC0 or CC BY 4.0 license, unless participant consent or institutional policy requires additional restrictions. Always ensure the selected license is consistent with participant consent and NIH/NIMH data sharing policies."
+  "1-Suggested file formats for each data type": {
+    "Demographic and Clinical Data": "CSV (Comma-Separated Values) or TSV (Tab-Separated Values). These are open, non-proprietary formats widely supported for tabular data, ensuring interoperability and long-term accessibility.",
+    "MRI and fMRI Imaging Data": "NIfTI (.nii or .nii.gz). NIfTI is the community standard for neuroimaging data, supporting interoperability and reuse.",
+    "1H fMRS Data": "NIfTI (.nii or .nii.gz) for imaging data; for raw spectroscopy data, use vendor-neutral formats such as LCModel (.RAW/.coord), jMRUI (.txt), or DICOM-MRS (if available). These formats are widely used and supported in the neuroimaging community.",
+    "Supporting Documentation": "PDF or plain text (.txt, .md) for protocols, README files, and data dictionaries to ensure accessibility and readability."
+  },
+  "2-Tools for converting data to the suggested file formats": {
+    "Demographic and Clinical Data": "Microsoft Excel, LibreOffice Calc, or R/Python scripts can export data to CSV/TSV.",
+    "MRI and fMRI Imaging Data": "dcm2niix for converting DICOM to NIfTI; SPM, FSL, or AFNI for further processing.",
+    "1H fMRS Data": "Vendor software (e.g., Siemens, Philips, GE) can export raw data; jMRUI, LCModel, or spec2nii can convert to open formats.",
+    "Supporting Documentation": "Any text editor (Notepad, VS Code) or word processor (Word, LibreOffice) for documentation files."
+  },
+  "3-Suggested standard structure to organize the dataset": "BIDS (Brain Imaging Data Structure) is the recommended standard for organizing neuroimaging datasets, including MRI, fMRI, and MRS data, as well as associated clinical and demographic information. BIDS ensures consistency, interoperability, and ease of reuse.",
+  "4-Tools for organizing the dataset in the suggested structure": "BIDS Starter Kit, HeuDiConv, bidskit, and the BIDS Validator can help organize and validate datasets according to the BIDS standard. The OpenNeuro platform also provides tools for BIDS-compliant dataset organization.",
+  "5-Metadata and information that should be provided with the data": "Comprehensive metadata should include: (1) Data dictionaries/codebooks for all variables; (2) README file describing the dataset, study design, and data collection protocols; (3) Protocols for imaging and clinical assessments; (4) BIDS-compliant JSON sidecar files for imaging data; (5) Data provenance and processing steps; (6) Consent language and IRB approval documentation (as appropriate for controlled access repositories).",
+  "6-Suggested standard structure and file format for metadata": "BIDS-compliant JSON files for imaging metadata; CSV/TSV for tabular data dictionaries; README and protocol files in plain text (.txt, .md) or PDF. For repository submission, follow the NIMH Data Archive (NDA) metadata requirements, which may include specific data dictionaries and manifest files.",
+  "7-Tools for preparing metadata in the suggested structure and file format": "BIDS Validator (web or command-line), BIDS Starter Kit templates, NDA Data Dictionary and Submission Tools, spreadsheet software for data dictionaries, and text editors for README/protocol files.",
+  "8-Suggested de-identification approach": "De-identification is required for all human subject data. All direct identifiers (names, dates of birth, addresses, etc.) must be removed. For imaging data, remove facial features from structural scans (defacing) and strip DICOM headers of identifying information. Collect and retain only the information necessary to generate the NIMH Data Archive (NDA) Global Unique Identifier (GUID). Since participants are consented for broad data sharing, data can be shared under controlled access with appropriate safeguards.",
+  "9-Tools to implement the suggested de-identification approach": "pydeface or mri_deface for defacing MRI images; dcm2niix for removing DICOM header information; NDA GUID Tool for generating subject identifiers; custom scripts or tools (e.g., ARX, Amnesia) for de-identifying tabular data.",
+  "10-Suggested repositories for sharing the dataset": "The NIMH Data Archive (NDA) is the required repository for NIMH-funded human subjects data. NDA supports controlled access, BIDS-compliant datasets, and the use of GUIDs for subject tracking. For additional open sharing of de-identified imaging data, OpenNeuro is a recommended secondary repository, provided all NDA requirements are met first.",
+  "11-Suggested license for sharing the dataset": "Data shared via NDA is subject to NDA's Data Use Certification and controlled access policies, which are designed to protect participant privacy while enabling broad scientific use. For secondary sharing (e.g., OpenNeuro), use the CC BY 4.0 license for de-identified data, unless further restrictions are required by consent or IRB. Always ensure that sharing complies with participant consent and institutional policies."
 }</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>For imaging data (MRI, 1H fMRS, fMRI), use NIfTI (.nii or .nii.gz) for volumetric data and BIDS-compliant formats for associated metadata (e.g., .json sidecars). For raw scanner data, DICOM (.dcm) may be retained but should be converted to NIfTI for sharing. For tabular data (demographics, clinical), use non-proprietary formats such as CSV (.csv) or TSV (.tsv). Documentation and metadata should be provided in plain text (.txt), Markdown (.md), or PDF (.pdf) formats. These formats are open, widely supported, and facilitate interoperability and reuse.</t>
+          <t>{'Demographic and Clinical Data': 'CSV (Comma-Separated Values) or TSV (Tab-Separated Values). These are open, non-proprietary formats widely supported for tabular data, ensuring interoperability and long-term accessibility.', 'MRI and fMRI Imaging Data': 'NIfTI (.nii or .nii.gz). NIfTI is the community standard for neuroimaging data, supporting interoperability and reuse.', '1H fMRS Data': 'NIfTI (.nii or .nii.gz) for imaging data; for raw spectroscopy data, use vendor-neutral formats such as LCModel (.RAW/.coord), jMRUI (.txt), or DICOM-MRS (if available). These formats are widely used and supported in the neuroimaging community.', 'Supporting Documentation': 'PDF or plain text (.txt, .md) for protocols, README files, and data dictionaries to ensure accessibility and readability.'}</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Use dcm2niix for DICOM to NIfTI conversion; BIDS Validator for checking dataset compliance; MRIQC and fMRIPrep for quality control and preprocessing; PyBIDS for programmatic BIDS data handling; spreadsheet software (e.g., Excel, LibreOffice) for tabular data (export as CSV/TSV); and Git or similar version control for tracking changes. For documentation, use text editors or Markdown tools.</t>
+          <t>{'Demographic and Clinical Data': 'Microsoft Excel, LibreOffice Calc, or R/Python scripts can export data to CSV/TSV.', 'MRI and fMRI Imaging Data': 'dcm2niix for converting DICOM to NIfTI; SPM, FSL, or AFNI for further processing.', '1H fMRS Data': 'Vendor software (e.g., Siemens, Philips, GE) can export raw data; jMRUI, LCModel, or spec2nii can convert to open formats.', 'Supporting Documentation': 'Any text editor (Notepad, VS Code) or word processor (Word, LibreOffice) for documentation files.'}</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Follow the Brain Imaging Data Structure (BIDS) standard for organizing and describing MRI, fMRI, and fMRS data. For clinical and demographic data, use BIDS 'participants.tsv' and associated data dictionaries. BIDS is widely accepted in neuroimaging and required by many repositories, including the NIMH Data Archive (NDA).</t>
+          <t>BIDS (Brain Imaging Data Structure) is the recommended standard for organizing neuroimaging datasets, including MRI, fMRI, and MRS data, as well as associated clinical and demographic information. BIDS ensures consistency, interoperability, and ease of reuse.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Organize data in a BIDS-compliant folder structure: a root directory with subfolders for each subject (e.g., sub-&lt;NDA_GUID&gt;), session folders if applicable, and modality-specific folders (anat, func, fmap, mrs, etc.). Use standardized BIDS file naming conventions (e.g., sub-&lt;NDA_GUID&gt;_ses-01_task-rest_bold.nii.gz). Store tabular data (demographics, clinical) in 'participants.tsv' and additional .tsv files as needed, with accompanying data dictionaries. Include a top-level README, dataset_description.json, and CHANGES file for versioning. Use consistent versioning for dataset updates and document changes in the CHANGES file.</t>
+          <t>BIDS Starter Kit, HeuDiConv, bidskit, and the BIDS Validator can help organize and validate datasets according to the BIDS standard. The OpenNeuro platform also provides tools for BIDS-compliant dataset organization.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Include a README file describing the dataset, a dataset_description.json (per BIDS), participants.tsv (with data dictionary), and modality-specific .json sidecar files for imaging data. Provide a data dictionary/codebook for all tabular data, protocols for data collection and processing, and a CHANGES file for version history. If using NDA, include NDA-specific metadata files as required.</t>
+          <t>Comprehensive metadata should include: (1) Data dictionaries/codebooks for all variables; (2) README file describing the dataset, study design, and data collection protocols; (3) Protocols for imaging and clinical assessments; (4) BIDS-compliant JSON sidecar files for imaging data; (5) Data provenance and processing steps; (6) Consent language and IRB approval documentation (as appropriate for controlled access repositories).</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Use the BIDS Validator (web or command-line) to check dataset and metadata compliance. The NDA Data Dictionary Tool can help prepare NDA-compliant metadata. For general metadata, tools like DataLad or CEDAR Workbench can assist with metadata management. Use spreadsheet software for data dictionaries, ensuring export to open formats.</t>
+          <t>BIDS-compliant JSON files for imaging metadata; CSV/TSV for tabular data dictionaries; README and protocol files in plain text (.txt, .md) or PDF. For repository submission, follow the NIMH Data Archive (NDA) metadata requirements, which may include specific data dictionaries and manifest files.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>De-identification is required for all human subjects data. Remove all direct identifiers from imaging and tabular data. For imaging, use tools like pydeface or mri_deface to remove facial features from structural scans. Ensure no PHI remains in DICOM headers or tabular files. Collect and use the NDA Global Unique Identifier (GUID) for each subject to enable linkage without direct identifiers. Since participants are consented for broad data sharing, data can be shared in accordance with NIH and NDA policies, but always confirm that consent language aligns with intended sharing scope.</t>
+          <t>BIDS Validator (web or command-line), BIDS Starter Kit templates, NDA Data Dictionary and Submission Tools, spreadsheet software for data dictionaries, and text editors for README/protocol files.</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Deposit all data in the NIMH Data Archive (NDA), as required for NIMH-funded human subjects research. NDA supports BIDS and provides infrastructure for secure, compliant sharing of deidentified human neuroimaging and associated data. Optionally, consider secondary sharing in OpenNeuro for broader community access, provided all NDA and consent requirements are met.</t>
+          <t>De-identification is required for all human subject data. All direct identifiers (names, dates of birth, addresses, etc.) must be removed. For imaging data, remove facial features from structural scans (defacing) and strip DICOM headers of identifying information. Collect and retain only the information necessary to generate the NIMH Data Archive (NDA) Global Unique Identifier (GUID). Since participants are consented for broad data sharing, data can be shared under controlled access with appropriate safeguards.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>For NDA, data are shared under NDA's Data Use Certification, which governs access and reuse. If sharing in additional repositories (e.g., OpenNeuro), use the Creative Commons CC0 or CC BY 4.0 license, unless participant consent or institutional policy requires additional restrictions. Always ensure the selected license is consistent with participant consent and NIH/NIMH data sharing policies.</t>
+          <t>pydeface or mri_deface for defacing MRI images; dcm2niix for removing DICOM header information; NDA GUID Tool for generating subject identifiers; custom scripts or tools (e.g., ARX, Amnesia) for de-identifying tabular data.</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>The NIMH Data Archive (NDA) is the required repository for NIMH-funded human subjects data. NDA supports controlled access, BIDS-compliant datasets, and the use of GUIDs for subject tracking. For additional open sharing of de-identified imaging data, OpenNeuro is a recommended secondary repository, provided all NDA requirements are met first.</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Data shared via NDA is subject to NDA's Data Use Certification and controlled access policies, which are designed to protect participant privacy while enabling broad scientific use. For secondary sharing (e.g., OpenNeuro), use the CC BY 4.0 license for de-identified data, unless further restrictions are required by consent or IRB. Always ensure that sharing complies with participant consent and institutional policies.</t>
         </is>
       </c>
     </row>
@@ -713,24 +751,28 @@
  will be submitted to the NIMH Data Archive (NDA). Phenotypic and clinical data for all 500 research subjects will 
  be collected and deposited in NDA using the data dictionaries available in NDA (described below).
 Based on these inputs, provide clear, practical, and user-friendly FAIR data guidance organized under the following sections:
-1. Recommended file formats
-Explain which file format(s) should be used for this type of data and why they are appropriate for FAIR sharing and reuse.
-2. Relevant tools and software
-List tools, software, or platforms that can help prepare, convert, validate, organize, document, or share this type of data.
-3. Recommended dataset structure or standard
-State the dataset structure, schema, or community standard that should be followed, if one exists.
-4. Dataset organization details
-Provide detailed guidance on how the dataset should be organized, including folder structure, file naming conventions, table organization, metadata arrangement, versioning considerations, and any other important technical details.
-5. Metadata and documentation files to include
-List the metadata files, README files, data dictionaries, codebooks, protocols, or other documentation that should accompany the dataset.
-6. Tools for metadata preparation and validation
-Suggest tools that can help create, validate, manage, or standardize metadata for this dataset.
-7. De-identification and privacy considerations
-State whether de-identification is required. Explain what should be done based on the subject type, the data modality, and whether the study involves human participants. If consent language affects sharing, explain that clearly.
-8. Recommended repositories
-Suggest appropriate repositories for sharing the data, prioritizing repositories recommended, required, or commonly accepted by the funding source and data type.
-9. Recommended data licenses
-Recommend appropriate data license(s), prioritizing those expected, suggested, or required by the funding source. If restrictions apply because of human subjects or consent limitations, explain that clearly.
+1- Suggested file formats for each data type
+Identify the recommended file format or formats for each data type in the dataset. Briefly explain why these formats are appropriate for FAIR sharing, reuse, interoperability, and long-term preservation.
+2- Tools for converting data to the suggested file formats
+List tools, software, or workflows that can be used to convert raw or source data into the recommended file formats.
+3- Suggested standard structure to organize the dataset
+State the recommended dataset structure, schema, specification, or community standard that should be used to organize the dataset, if one exists.
+4- Tools for organizing the dataset in the suggested structure
+List tools, software, templates, or platforms that can help organize the dataset according to the recommended structure or standard.
+5- Metadata and information that should be provided with the data
+Describe the metadata, documentation, contextual information, data dictionaries, codebooks, README files, protocols, and any other supporting information that should accompany the dataset.
+6- Suggested standard structure and file format for metadata
+State the recommended structure, schema, standard, and file format that should be used for metadata and documentation files included with the dataset.
+7-Tools for preparing metadata in the suggested structure and file format
+List tools, software, validators, templates, or platforms that can help create, manage, standardize, or validate metadata in the recommended structure and format.
+8- Suggested de-identification approach
+State whether de-identification is required. Explain the recommended de-identification or privacy-preserving approach based on the subject type, data modality, sensitivity of the data, and whether human participants are involved. If consent language affects sharing, explain that clearly.
+9- Tools to implement the suggested de-identification approach
+List tools, software, workflows, or methods that can help implement the recommended de-identification or privacy protection approach.
+10-Suggested repositories for sharing the dataset
+Recommend appropriate repositories for sharing the dataset, prioritizing repositories required, recommended, or commonly accepted by the funding source, subject type, and data modality.
+11- Suggested license for sharing the dataset
+Recommend an appropriate data license or licensing approach, prioritizing what is expected, suggested, or required by the funding source. If restrictions apply because of human subjects, controlled access, or consent limitations, explain that clearly.
 Instructions for your response:
 - Make the guidance practical, concise, and easy for researchers to follow.
 - Tailor all recommendations to the combination of funding source, human-subject status, consent language, and data modality.
@@ -741,76 +783,99 @@
 Return your answer in valid JSON format only.
 Use exactly this JSON structure:
 {
-  "Recommended file formats": "",
-  "Relevant tools and software": "",
-  "Recommended dataset structure or standard": "",
-  "Dataset organization details": "",
-  "Metadata and documentation files to include": "",
-  "Tools for metadata preparation and validation": "",
-  "De-identification and privacy considerations": "",
-  "Recommended repositories": "",
-  "Recommended data licenses": ""
+  "1-Suggested file formats for each data type": "",
+  "2-Tools for converting data to the suggested file formats": "",
+  "3-Suggested standard structure to organize the dataset": "",
+  "4-Tools for organizing the dataset in the suggested structure": "",
+  "5-Metadata and information that should be provided with the data": "",
+  "6-Suggested standard structure and file format for metadata": "",
+  "7-Tools for preparing metadata in the suggested structure and file format": "",
+  "8-Suggested de-identification approach": "",
+  "9-Tools to implement the suggested de-identification approach": "",
+  "10-Suggested repositories for sharing the dataset": "",
+  "11-Suggested license for sharing the dataset": ""
 }</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
           <t>{
-  "Recommended file formats": "For raw whole genome sequencing (WGS) data, use FASTQ for raw reads and BAM/CRAM for aligned reads, as these are standard, widely supported, and required by dbGaP and NDA. For variant data, use VCF (Variant Call Format). For phenotypic and clinical data, use CSV or TSV files structured according to NDA data dictionaries. Metadata should be provided in machine-readable formats such as XML or JSON, as required by the repository.",
-  "Relevant tools and software": "Use bcl2fastq or Illumina BaseSpace for FASTQ generation; SAMtools or Picard for BAM/CRAM processing; GATK for variant calling and VCF generation. For phenotypic data, use spreadsheet software (Excel, Google Sheets) for initial entry, then export to CSV/TSV. NDA provides the Data Dictionary Tool and Validation Tool for formatting and validating submissions. dbGaP provides submission tools and templates. For metadata, use tools like ISA-Tab or the NDA's own metadata submission interface.",
-  "Recommended dataset structure or standard": "Follow the NIMH Data Archive (NDA) data dictionary and schema for phenotypic and clinical data. For genomic data, adhere to dbGaP and NDA submission guidelines, which specify file formats and metadata requirements. Use the NIH Genomic Data Sharing (GDS) Policy as an overarching standard. For metadata, use the MIABIS (Minimum Information About BIobank data Sharing) or MIAME (for microarray data, if applicable) standards as references.",
-  "Dataset organization details": "Organize data in a hierarchical folder structure: /raw_data/ (FASTQ, BAM/CRAM), /variants/ (VCF), /phenotype/ (CSV/TSV per NDA dictionary), /metadata/ (README, data dictionary, consent forms), /docs/ (protocols, codebooks). Use clear, consistent file naming conventions: [studyID]_[datatype]_[subjectID]_[date].[ext] (e.g., ABC123_WGS_001_20240601.bam). Each table should have a header row matching NDA data dictionary fields. Maintain a version log (CHANGELOG.txt) and use versioned folders or file suffixes for updates. Ensure all files are referenced in a master README.",
-  "Metadata and documentation files to include": "Include a comprehensive README.txt describing the dataset, data collection methods, and file structure. Provide data dictionaries for all phenotypic/clinical tables (as per NDA requirements), codebooks explaining variable meanings, and protocols for sample collection and sequencing. Include consent form templates and IRB approval documentation. Provide a manifest file listing all files and their checksums. Include submission metadata files required by dbGaP and NDA.",
-  "Tools for metadata preparation and validation": "Use the NDA Data Dictionary Tool and Validation Tool for preparing and checking phenotypic/clinical data. dbGaP provides metadata templates and validation scripts. For general metadata, use ISA-Tab tools or spreadsheet-to-JSON/XML converters. Consider using OpenRefine for data cleaning and standardization.",
-  "De-identification and privacy considerations": "De-identification is required for all human subject data. Remove all direct identifiers (names, addresses, contact info) and use NDA Global Unique Identifiers (GUIDs) for subject tracking. Ensure dates are offset or generalized as per NDA/dbGaP guidelines. Since participants are consented for broad data sharing, data can be shared via controlled-access repositories (dbGaP, NDA) in compliance with NIH Genomic Data Sharing Policy. Include a description of de-identification procedures in your documentation.",
-  "Recommended repositories": "Submit raw and processed genomic data to dbGaP (as required by NIH for genomic data) and to the NIMH Data Archive (NDA) for both genomic and phenotypic/clinical data, following their submission guidelines. These repositories are NIH-recommended and meet NIMH expectations for data sharing.",
-  "Recommended data licenses": "For human genomic and phenotypic data, use the NIH Genomic Data Sharing Policy's controlled-access model. Data will not have an open license but will be shared under dbGaP and NDA Data Use Certifications, which restrict use to approved researchers and projects. Clearly state in documentation that data access is controlled due to human subject protections, even with broad consent."
+  "1-Suggested file formats for each data type": {
+    "Genomic raw data": "FASTQ (raw reads), BAM/CRAM (aligned reads), and VCF (variant calls). These are community-standard, open formats widely supported for genomic data sharing, analysis, and long-term preservation.",
+    "Derived genomic data": "VCF for variant calls, and tab-delimited text (TSV/CSV) for summary statistics. These formats are interoperable and facilitate downstream reuse.",
+    "Phenotypic and clinical data": "Tab-delimited text (TSV) or comma-separated values (CSV), structured according to NDA data dictionary templates. These formats are machine-readable, open, and support interoperability.",
+    "Supporting documentation": "PDF or plain text (TXT/Markdown) for protocols, README, and codebooks. These formats are accessible and preserve formatting."
+  },
+  "2-Tools for converting data to the suggested file formats": {
+    "Genomic data": "bcl2fastq (Illumina), samtools (for BAM/CRAM), GATK or bcftools (for VCF).",
+    "Phenotypic/clinical data": "Spreadsheet software (Excel, Google Sheets) for initial entry, then export as CSV/TSV. NDA Data Dictionary Tool for formatting to NDA standards.",
+    "Documentation": "Word processors (MS Word, Google Docs) for authoring, then export as PDF or TXT."
+  },
+  "3-Suggested standard structure to organize the dataset": "Follow the NIMH Data Archive (NDA) data structure, which requires data to be organized according to NDA data dictionaries and submission guidelines. For genomic data, follow dbGaP submission structure, which includes separate folders for raw data, processed data, and metadata.",
+  "4-Tools for organizing the dataset in the suggested structure": "NDA Data Submission Tool (NDA Upload Tool), NDA Data Dictionary Tool, dbGaP Submission Portal, and file organization scripts (e.g., Python, R, or shell scripts) to structure files and folders as required.",
+  "5-Metadata and information that should be provided with the data": "Comprehensive metadata including study description, data collection protocols, consent language, subject-level data dictionaries, variable definitions, codebooks, README files describing file contents and structure, data provenance, and any data processing or QC steps. For NDA, use the required data dictionary and data element definitions. For dbGaP, provide study documentation, sample attributes, and data processing details.",
+  "6-Suggested standard structure and file format for metadata": "NDA requires metadata in their standardized data dictionary format (CSV/TSV) and study-level metadata in XML or web forms. dbGaP requires metadata in XML and tabular formats as per their submission guidelines. README and protocols should be in PDF or TXT.",
+  "7-Tools for preparing metadata in the suggested structure and file format": "NDA Data Dictionary Tool, NDA web-based metadata entry forms, dbGaP Submission Portal, and metadata validators provided by NDA and dbGaP. Spreadsheet software for preparing tabular metadata, and text editors for documentation files.",
+  "8-Suggested de-identification approach": "De-identification is required for all human subject data. Remove all direct identifiers (names, addresses, contact information, etc.) and use NDA Global Unique Identifiers (GUIDs) for subject tracking. For genomic data, follow dbGaP and NDA guidelines for de-identification, ensuring no residual identifiers remain. Since broad data sharing consent is obtained, data can be shared under controlled access with appropriate privacy safeguards.",
+  "9-Tools to implement the suggested de-identification approach": "NDA GUID Tool for generating subject identifiers, NDA Data Validation and De-identification Tools, dbGaP de-identification checklists, and custom scripts for removing identifiers from datasets.",
+  "10-Suggested repositories for sharing the dataset": "Raw and processed genomic data: dbGaP (required by NIH for human genomic data). Phenotypic, clinical, and derived data: NIMH Data Archive (NDA), as required by NIMH. Both repositories support controlled access and are compliant with NIH data sharing policies.",
+  "11-Suggested license for sharing the dataset": "Data should be shared under controlled access as required by NIH and NIMH for human subject data, with data use agreements specifying permitted uses. No open/public license is permitted for identifiable or potentially re-identifiable human data. Reference the NIH Genomic Data Sharing Policy and NDA Data Use Terms in documentation."
 }</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>For raw whole genome sequencing (WGS) data, use FASTQ for raw reads and BAM/CRAM for aligned reads, as these are standard, widely supported, and required by dbGaP and NDA. For variant data, use VCF (Variant Call Format). For phenotypic and clinical data, use CSV or TSV files structured according to NDA data dictionaries. Metadata should be provided in machine-readable formats such as XML or JSON, as required by the repository.</t>
+          <t>{'Genomic raw data': 'FASTQ (raw reads), BAM/CRAM (aligned reads), and VCF (variant calls). These are community-standard, open formats widely supported for genomic data sharing, analysis, and long-term preservation.', 'Derived genomic data': 'VCF for variant calls, and tab-delimited text (TSV/CSV) for summary statistics. These formats are interoperable and facilitate downstream reuse.', 'Phenotypic and clinical data': 'Tab-delimited text (TSV) or comma-separated values (CSV), structured according to NDA data dictionary templates. These formats are machine-readable, open, and support interoperability.', 'Supporting documentation': 'PDF or plain text (TXT/Markdown) for protocols, README, and codebooks. These formats are accessible and preserve formatting.'}</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Use bcl2fastq or Illumina BaseSpace for FASTQ generation; SAMtools or Picard for BAM/CRAM processing; GATK for variant calling and VCF generation. For phenotypic data, use spreadsheet software (Excel, Google Sheets) for initial entry, then export to CSV/TSV. NDA provides the Data Dictionary Tool and Validation Tool for formatting and validating submissions. dbGaP provides submission tools and templates. For metadata, use tools like ISA-Tab or the NDA's own metadata submission interface.</t>
+          <t>{'Genomic data': 'bcl2fastq (Illumina), samtools (for BAM/CRAM), GATK or bcftools (for VCF).', 'Phenotypic/clinical data': 'Spreadsheet software (Excel, Google Sheets) for initial entry, then export as CSV/TSV. NDA Data Dictionary Tool for formatting to NDA standards.', 'Documentation': 'Word processors (MS Word, Google Docs) for authoring, then export as PDF or TXT.'}</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Follow the NIMH Data Archive (NDA) data dictionary and schema for phenotypic and clinical data. For genomic data, adhere to dbGaP and NDA submission guidelines, which specify file formats and metadata requirements. Use the NIH Genomic Data Sharing (GDS) Policy as an overarching standard. For metadata, use the MIABIS (Minimum Information About BIobank data Sharing) or MIAME (for microarray data, if applicable) standards as references.</t>
+          <t>Follow the NIMH Data Archive (NDA) data structure, which requires data to be organized according to NDA data dictionaries and submission guidelines. For genomic data, follow dbGaP submission structure, which includes separate folders for raw data, processed data, and metadata.</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Organize data in a hierarchical folder structure: /raw_data/ (FASTQ, BAM/CRAM), /variants/ (VCF), /phenotype/ (CSV/TSV per NDA dictionary), /metadata/ (README, data dictionary, consent forms), /docs/ (protocols, codebooks). Use clear, consistent file naming conventions: [studyID]_[datatype]_[subjectID]_[date].[ext] (e.g., ABC123_WGS_001_20240601.bam). Each table should have a header row matching NDA data dictionary fields. Maintain a version log (CHANGELOG.txt) and use versioned folders or file suffixes for updates. Ensure all files are referenced in a master README.</t>
+          <t>NDA Data Submission Tool (NDA Upload Tool), NDA Data Dictionary Tool, dbGaP Submission Portal, and file organization scripts (e.g., Python, R, or shell scripts) to structure files and folders as required.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Include a comprehensive README.txt describing the dataset, data collection methods, and file structure. Provide data dictionaries for all phenotypic/clinical tables (as per NDA requirements), codebooks explaining variable meanings, and protocols for sample collection and sequencing. Include consent form templates and IRB approval documentation. Provide a manifest file listing all files and their checksums. Include submission metadata files required by dbGaP and NDA.</t>
+          <t>Comprehensive metadata including study description, data collection protocols, consent language, subject-level data dictionaries, variable definitions, codebooks, README files describing file contents and structure, data provenance, and any data processing or QC steps. For NDA, use the required data dictionary and data element definitions. For dbGaP, provide study documentation, sample attributes, and data processing details.</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Use the NDA Data Dictionary Tool and Validation Tool for preparing and checking phenotypic/clinical data. dbGaP provides metadata templates and validation scripts. For general metadata, use ISA-Tab tools or spreadsheet-to-JSON/XML converters. Consider using OpenRefine for data cleaning and standardization.</t>
+          <t>NDA requires metadata in their standardized data dictionary format (CSV/TSV) and study-level metadata in XML or web forms. dbGaP requires metadata in XML and tabular formats as per their submission guidelines. README and protocols should be in PDF or TXT.</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>De-identification is required for all human subject data. Remove all direct identifiers (names, addresses, contact info) and use NDA Global Unique Identifiers (GUIDs) for subject tracking. Ensure dates are offset or generalized as per NDA/dbGaP guidelines. Since participants are consented for broad data sharing, data can be shared via controlled-access repositories (dbGaP, NDA) in compliance with NIH Genomic Data Sharing Policy. Include a description of de-identification procedures in your documentation.</t>
+          <t>NDA Data Dictionary Tool, NDA web-based metadata entry forms, dbGaP Submission Portal, and metadata validators provided by NDA and dbGaP. Spreadsheet software for preparing tabular metadata, and text editors for documentation files.</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Submit raw and processed genomic data to dbGaP (as required by NIH for genomic data) and to the NIMH Data Archive (NDA) for both genomic and phenotypic/clinical data, following their submission guidelines. These repositories are NIH-recommended and meet NIMH expectations for data sharing.</t>
+          <t>De-identification is required for all human subject data. Remove all direct identifiers (names, addresses, contact information, etc.) and use NDA Global Unique Identifiers (GUIDs) for subject tracking. For genomic data, follow dbGaP and NDA guidelines for de-identification, ensuring no residual identifiers remain. Since broad data sharing consent is obtained, data can be shared under controlled access with appropriate privacy safeguards.</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>For human genomic and phenotypic data, use the NIH Genomic Data Sharing Policy's controlled-access model. Data will not have an open license but will be shared under dbGaP and NDA Data Use Certifications, which restrict use to approved researchers and projects. Clearly state in documentation that data access is controlled due to human subject protections, even with broad consent.</t>
+          <t>NDA GUID Tool for generating subject identifiers, NDA Data Validation and De-identification Tools, dbGaP de-identification checklists, and custom scripts for removing identifiers from datasets.</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Raw and processed genomic data: dbGaP (required by NIH for human genomic data). Phenotypic, clinical, and derived data: NIMH Data Archive (NDA), as required by NIMH. Both repositories support controlled access and are compliant with NIH data sharing policies.</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Data should be shared under controlled access as required by NIH and NIMH for human subject data, with data use agreements specifying permitted uses. No open/public license is permitted for identifiable or potentially re-identifiable human data. Reference the NIH Genomic Data Sharing Policy and NDA Data Use Terms in documentation.</t>
         </is>
       </c>
     </row>
@@ -875,24 +940,28 @@
  The amount and type of data from human cells will depend on the results from the mouse studies. Data sharing 
  plans will be updated when appropriate (likely at the start of year 4 of the grant award).
 Based on these inputs, provide clear, practical, and user-friendly FAIR data guidance organized under the following sections:
-1. Recommended file formats
-Explain which file format(s) should be used for this type of data and why they are appropriate for FAIR sharing and reuse.
-2. Relevant tools and software
-List tools, software, or platforms that can help prepare, convert, validate, organize, document, or share this type of data.
-3. Recommended dataset structure or standard
-State the dataset structure, schema, or community standard that should be followed, if one exists.
-4. Dataset organization details
-Provide detailed guidance on how the dataset should be organized, including folder structure, file naming conventions, table organization, metadata arrangement, versioning considerations, and any other important technical details.
-5. Metadata and documentation files to include
-List the metadata files, README files, data dictionaries, codebooks, protocols, or other documentation that should accompany the dataset.
-6. Tools for metadata preparation and validation
-Suggest tools that can help create, validate, manage, or standardize metadata for this dataset.
-7. De-identification and privacy considerations
-State whether de-identification is required. Explain what should be done based on the subject type, the data modality, and whether the study involves human participants. If consent language affects sharing, explain that clearly.
-8. Recommended repositories
-Suggest appropriate repositories for sharing the data, prioritizing repositories recommended, required, or commonly accepted by the funding source and data type.
-9. Recommended data licenses
-Recommend appropriate data license(s), prioritizing those expected, suggested, or required by the funding source. If restrictions apply because of human subjects or consent limitations, explain that clearly.
+1- Suggested file formats for each data type
+Identify the recommended file format or formats for each data type in the dataset. Briefly explain why these formats are appropriate for FAIR sharing, reuse, interoperability, and long-term preservation.
+2- Tools for converting data to the suggested file formats
+List tools, software, or workflows that can be used to convert raw or source data into the recommended file formats.
+3- Suggested standard structure to organize the dataset
+State the recommended dataset structure, schema, specification, or community standard that should be used to organize the dataset, if one exists.
+4- Tools for organizing the dataset in the suggested structure
+List tools, software, templates, or platforms that can help organize the dataset according to the recommended structure or standard.
+5- Metadata and information that should be provided with the data
+Describe the metadata, documentation, contextual information, data dictionaries, codebooks, README files, protocols, and any other supporting information that should accompany the dataset.
+6- Suggested standard structure and file format for metadata
+State the recommended structure, schema, standard, and file format that should be used for metadata and documentation files included with the dataset.
+7-Tools for preparing metadata in the suggested structure and file format
+List tools, software, validators, templates, or platforms that can help create, manage, standardize, or validate metadata in the recommended structure and format.
+8- Suggested de-identification approach
+State whether de-identification is required. Explain the recommended de-identification or privacy-preserving approach based on the subject type, data modality, sensitivity of the data, and whether human participants are involved. If consent language affects sharing, explain that clearly.
+9- Tools to implement the suggested de-identification approach
+List tools, software, workflows, or methods that can help implement the recommended de-identification or privacy protection approach.
+10-Suggested repositories for sharing the dataset
+Recommend appropriate repositories for sharing the dataset, prioritizing repositories required, recommended, or commonly accepted by the funding source, subject type, and data modality.
+11- Suggested license for sharing the dataset
+Recommend an appropriate data license or licensing approach, prioritizing what is expected, suggested, or required by the funding source. If restrictions apply because of human subjects, controlled access, or consent limitations, explain that clearly.
 Instructions for your response:
 - Make the guidance practical, concise, and easy for researchers to follow.
 - Tailor all recommendations to the combination of funding source, human-subject status, consent language, and data modality.
@@ -903,76 +972,90 @@
 Return your answer in valid JSON format only.
 Use exactly this JSON structure:
 {
-  "Recommended file formats": "",
-  "Relevant tools and software": "",
-  "Recommended dataset structure or standard": "",
-  "Dataset organization details": "",
-  "Metadata and documentation files to include": "",
-  "Tools for metadata preparation and validation": "",
-  "De-identification and privacy considerations": "",
-  "Recommended repositories": "",
-  "Recommended data licenses": ""
+  "1-Suggested file formats for each data type": "",
+  "2-Tools for converting data to the suggested file formats": "",
+  "3-Suggested standard structure to organize the dataset": "",
+  "4-Tools for organizing the dataset in the suggested structure": "",
+  "5-Metadata and information that should be provided with the data": "",
+  "6-Suggested standard structure and file format for metadata": "",
+  "7-Tools for preparing metadata in the suggested structure and file format": "",
+  "8-Suggested de-identification approach": "",
+  "9-Tools to implement the suggested de-identification approach": "",
+  "10-Suggested repositories for sharing the dataset": "",
+  "11-Suggested license for sharing the dataset": ""
 }</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>{
-  "Recommended file formats": "For single-cell omics data (ATAC-seq, RNA-seq, DNA methylation) from mouse brain, use open, community-accepted formats: (1) Matrix data: Use Matrix Market (.mtx) or HDF5-based formats (e.g., .h5ad for AnnData, .loom for Loom files) for count matrices. (2) Metadata: Use tab-delimited text (.tsv) or comma-separated values (.csv) for cell and sample metadata tables. (3) Genomic ranges: Use BED (.bed) or BigBed for peak or region annotations. (4) Protocols and documentation: Use PDF or Markdown (.md). These formats are widely supported, interoperable, and facilitate reuse and sharing.",
-  "Relevant tools and software": "Recommended tools include: (1) Scanpy (Python) and Seurat (R) for single-cell data processing and export to .h5ad, .loom, or .csv/.tsv. (2) Cell Ranger (10x Genomics) for initial processing. (3) AnnData and Loompy for HDF5-based file handling. (4) UCSC tools or BEDTools for genomic interval files. (5) Data validation: Frictionless Data (for tabular data), HDFView (for HDF5 files). (6) Data organization and sharing: Globus, Synapse, or direct upload to repositories.",
-  "Recommended dataset structure or standard": "Follow the Human Cell Atlas (HCA) metadata schema and the Minimum Information About a Single Cell Experiment (MINISE) guidelines, adapted for mouse data. For spatial data, refer to the Spatial Omics Data Structure (SODS) or the OME-NGFF (Open Microscopy Environment Next-Generation File Format) for spatial coordinates. Organize data as per the Single Cell Expression Atlas or HCA conventions: separate files for count matrices, metadata, and feature annotations.",
-  "Dataset organization details": "Organize the dataset in a clear folder hierarchy: (1) /raw_data/ (raw sequencing files, e.g., FASTQ, if sharing), (2) /processed_data/ (count matrices in .mtx, .h5ad, or .loom), (3) /metadata/ (cell/sample metadata tables in .csv/.tsv), (4) /annotations/ (peak/gene/region files in .bed), (5) /docs/ (README, protocols, data dictionary). Use descriptive, consistent file naming: e.g., modality_species_stage_matrix.mtx, modality_species_stage_metadata.csv. Include version numbers in file names or a VERSION.txt file. Document all QC metrics and processing steps in the metadata and README. Ensure each cell and sample has a unique, stable identifier.",
-  "Metadata and documentation files to include": "Include: (1) README.txt or README.md describing dataset contents, structure, and usage; (2) Data dictionary/codebook explaining all columns in metadata tables; (3) Protocols (PDF or Markdown) detailing experimental and computational methods; (4) Sample and cell metadata files (.csv/.tsv) with all relevant attributes; (5) QC metrics summary; (6) VERSION.txt or changelog; (7) References to relevant standards or schema used.",
-  "Tools for metadata preparation and validation": "Use Frictionless Data's Table Schema or Goodtables for tabular metadata validation. The HCA Metadata Schema Validator (adapted for mouse) can help ensure compliance with community standards. For spatial metadata, use OME-NGFF tools. Consider using ISA-Tab or CEDAR Workbench for structured metadata entry and validation.",
-  "De-identification and privacy considerations": "No human subjects are involved in the current dataset; therefore, de-identification is not required for mouse data. If human data are added in the future, follow NIH and NIMH policies: remove all direct and indirect identifiers, ensure data are de-identified to HIPAA standards, and confirm that consent language permits data sharing. Update the data sharing plan and repository selection accordingly.",
-  "Recommended repositories": "For mouse single-cell omics data, deposit in the NIMH Data Archive (NDA) if required by NIMH, or in community repositories such as Gene Expression Omnibus (GEO), ArrayExpress, or Single Cell Expression Atlas. For spatial omics, consider the Brain Image Library (BIL) or the Single Cell Portal (Broad Institute). If data are multi-modal or spatial, ensure the repository supports these formats. Provide persistent identifiers (e.g., accession numbers, DOIs) in publications.",
-  "Recommended data licenses": "NIH strongly encourages open data sharing. Use the Creative Commons CC0 1.0 Universal (Public Domain Dedication) license for mouse data, as recommended by NIH and major repositories (e.g., GEO, ArrayExpress). If future human data are subject to consent or privacy restrictions, select a license that aligns with those constraints and update documentation accordingly."
+  "1-Suggested file formats for each data type": "For single-cell matrices (ATAC, RNA, DNAm): use Matrix Market (.mtx), HDF5 (.h5ad for AnnData, .h5 for loom), or CSV/TSV for smaller datasets. For metadata tables: use CSV or TSV. These formats are widely supported, open, and facilitate interoperability, reuse, and long-term preservation. For spatial coordinates and punch information, include as columns in the metadata table or as a separate CSV/TSV file. For QC metrics, include as columns in the metadata table.",
+  "2-Tools for converting data to the suggested file formats": "Seurat (R), Scanpy (Python), and Bioconductor packages (e.g., SingleCellExperiment, scater) can export data to .mtx, .h5ad, .loom, and CSV/TSV. For ATAC-seq, ArchR and Signac support export to these formats. For methylation data, methylKit and bsseq can export to CSV/TSV. Standard spreadsheet software (Excel, LibreOffice) can export metadata tables to CSV/TSV.",
+  "3-Suggested standard structure to organize the dataset": "Recommended approach: Use the Human Cell Atlas (HCA) data structure or the Open Biological and Biomedical Ontology (OBO) Foundry standards for single-cell data. Organize data by modality (e.g., /RNA/, /ATAC/, /DNAm/), with subfolders for matrices, metadata, and QC. Follow the Single Cell Expression Atlas and HCA conventions for file naming and folder organization.",
+  "4-Tools for organizing the dataset in the suggested structure": "The HCA Data Coordination Platform (DCP) tools, Single Cell Expression Atlas submission templates, and the nf-core/scrnaseq pipeline can help structure data. Custom scripts (Python, R) and workflow managers (Snakemake, Nextflow) can automate organization. The DataLad and BIDS Starter Kit can assist with reproducible dataset structuring.",
+  "5-Metadata and information that should be provided with the data": "Provide a comprehensive README file describing the dataset, study design, and data processing steps. Include a data dictionary/codebook for all metadata fields. Supply protocols for sample preparation, sequencing, and QC. Document all variables (e.g., animal sex, developmental time point, punch coordinates, cluster assignments, QC metrics). Include software versions and parameter settings. Reference relevant ontologies (e.g., Cell Ontology, Uberon for anatomical terms).",
+  "6-Suggested standard structure and file format for metadata": "Recommended approach: Use the Minimum Information About a Single Cell Experiment (MINISE) or HCA metadata schema, provided as JSON or TSV/CSV. For general dataset description, use DataCite or schema.org metadata in JSON-LD. README and protocols should be in plain text or PDF. Data dictionaries should be in CSV/TSV or Markdown.",
+  "7-Tools for preparing metadata in the suggested structure and file format": "HCA metadata submission tools, DataCite Metadata Generator, schema.org JSON-LD generators, and the Single Cell Expression Atlas metadata templates. Spreadsheet software for CSV/TSV. The BioSamples metadata validator and FAIRsharing registry can help validate metadata. Protocols.io can be used for protocol documentation.",
+  "8-Suggested de-identification approach": "De-identification is not required for mouse data, as no human subjects are involved in the initial dataset. If human data are added in the future, follow NIH and NIMH policies: remove all direct and indirect identifiers, and ensure data are shared in accordance with consent and IRB requirements. Update the data sharing plan accordingly.",
+  "9-Tools to implement the suggested de-identification approach": "For mouse data, no de-identification tools are needed. For future human data, use tools such as the NIMH Data Archive (NDA) de-identification guidance, the HIPAA Safe Harbor checklist, and the Open Brain Consent de-identification scripts for omics data.",
+  "10-Suggested repositories for sharing the dataset": "For mouse single-cell omics data, deposit in the Gene Expression Omnibus (GEO) or ArrayExpress for general omics data, and the Single Cell Expression Atlas for single-cell data. For spatial transcriptomics, consider the Brain Image Library (BIL) or the Neuroscience Multi-Omic Archive (NeMO). NIH strongly encourages use of these repositories. If human data are added, use controlled-access repositories such as dbGaP or the NIMH Data Archive (NDA) as appropriate.",
+  "11-Suggested license for sharing the dataset": "Recommended approach: Use the Creative Commons Attribution 4.0 International (CC BY 4.0) license, which is NIH- and NIMH-compliant and maximizes reuse. If human data are added and consent restricts sharing, use a more restrictive license or controlled-access terms as required by the consent and IRB."
 }</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>For single-cell omics data (ATAC-seq, RNA-seq, DNA methylation) from mouse brain, use open, community-accepted formats: (1) Matrix data: Use Matrix Market (.mtx) or HDF5-based formats (e.g., .h5ad for AnnData, .loom for Loom files) for count matrices. (2) Metadata: Use tab-delimited text (.tsv) or comma-separated values (.csv) for cell and sample metadata tables. (3) Genomic ranges: Use BED (.bed) or BigBed for peak or region annotations. (4) Protocols and documentation: Use PDF or Markdown (.md). These formats are widely supported, interoperable, and facilitate reuse and sharing.</t>
+          <t>For single-cell matrices (ATAC, RNA, DNAm): use Matrix Market (.mtx), HDF5 (.h5ad for AnnData, .h5 for loom), or CSV/TSV for smaller datasets. For metadata tables: use CSV or TSV. These formats are widely supported, open, and facilitate interoperability, reuse, and long-term preservation. For spatial coordinates and punch information, include as columns in the metadata table or as a separate CSV/TSV file. For QC metrics, include as columns in the metadata table.</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Recommended tools include: (1) Scanpy (Python) and Seurat (R) for single-cell data processing and export to .h5ad, .loom, or .csv/.tsv. (2) Cell Ranger (10x Genomics) for initial processing. (3) AnnData and Loompy for HDF5-based file handling. (4) UCSC tools or BEDTools for genomic interval files. (5) Data validation: Frictionless Data (for tabular data), HDFView (for HDF5 files). (6) Data organization and sharing: Globus, Synapse, or direct upload to repositories.</t>
+          <t>Seurat (R), Scanpy (Python), and Bioconductor packages (e.g., SingleCellExperiment, scater) can export data to .mtx, .h5ad, .loom, and CSV/TSV. For ATAC-seq, ArchR and Signac support export to these formats. For methylation data, methylKit and bsseq can export to CSV/TSV. Standard spreadsheet software (Excel, LibreOffice) can export metadata tables to CSV/TSV.</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Follow the Human Cell Atlas (HCA) metadata schema and the Minimum Information About a Single Cell Experiment (MINISE) guidelines, adapted for mouse data. For spatial data, refer to the Spatial Omics Data Structure (SODS) or the OME-NGFF (Open Microscopy Environment Next-Generation File Format) for spatial coordinates. Organize data as per the Single Cell Expression Atlas or HCA conventions: separate files for count matrices, metadata, and feature annotations.</t>
+          <t>Recommended approach: Use the Human Cell Atlas (HCA) data structure or the Open Biological and Biomedical Ontology (OBO) Foundry standards for single-cell data. Organize data by modality (e.g., /RNA/, /ATAC/, /DNAm/), with subfolders for matrices, metadata, and QC. Follow the Single Cell Expression Atlas and HCA conventions for file naming and folder organization.</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Organize the dataset in a clear folder hierarchy: (1) /raw_data/ (raw sequencing files, e.g., FASTQ, if sharing), (2) /processed_data/ (count matrices in .mtx, .h5ad, or .loom), (3) /metadata/ (cell/sample metadata tables in .csv/.tsv), (4) /annotations/ (peak/gene/region files in .bed), (5) /docs/ (README, protocols, data dictionary). Use descriptive, consistent file naming: e.g., modality_species_stage_matrix.mtx, modality_species_stage_metadata.csv. Include version numbers in file names or a VERSION.txt file. Document all QC metrics and processing steps in the metadata and README. Ensure each cell and sample has a unique, stable identifier.</t>
+          <t>The HCA Data Coordination Platform (DCP) tools, Single Cell Expression Atlas submission templates, and the nf-core/scrnaseq pipeline can help structure data. Custom scripts (Python, R) and workflow managers (Snakemake, Nextflow) can automate organization. The DataLad and BIDS Starter Kit can assist with reproducible dataset structuring.</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Include: (1) README.txt or README.md describing dataset contents, structure, and usage; (2) Data dictionary/codebook explaining all columns in metadata tables; (3) Protocols (PDF or Markdown) detailing experimental and computational methods; (4) Sample and cell metadata files (.csv/.tsv) with all relevant attributes; (5) QC metrics summary; (6) VERSION.txt or changelog; (7) References to relevant standards or schema used.</t>
+          <t>Provide a comprehensive README file describing the dataset, study design, and data processing steps. Include a data dictionary/codebook for all metadata fields. Supply protocols for sample preparation, sequencing, and QC. Document all variables (e.g., animal sex, developmental time point, punch coordinates, cluster assignments, QC metrics). Include software versions and parameter settings. Reference relevant ontologies (e.g., Cell Ontology, Uberon for anatomical terms).</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Use Frictionless Data's Table Schema or Goodtables for tabular metadata validation. The HCA Metadata Schema Validator (adapted for mouse) can help ensure compliance with community standards. For spatial metadata, use OME-NGFF tools. Consider using ISA-Tab or CEDAR Workbench for structured metadata entry and validation.</t>
+          <t>Recommended approach: Use the Minimum Information About a Single Cell Experiment (MINISE) or HCA metadata schema, provided as JSON or TSV/CSV. For general dataset description, use DataCite or schema.org metadata in JSON-LD. README and protocols should be in plain text or PDF. Data dictionaries should be in CSV/TSV or Markdown.</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>No human subjects are involved in the current dataset; therefore, de-identification is not required for mouse data. If human data are added in the future, follow NIH and NIMH policies: remove all direct and indirect identifiers, ensure data are de-identified to HIPAA standards, and confirm that consent language permits data sharing. Update the data sharing plan and repository selection accordingly.</t>
+          <t>HCA metadata submission tools, DataCite Metadata Generator, schema.org JSON-LD generators, and the Single Cell Expression Atlas metadata templates. Spreadsheet software for CSV/TSV. The BioSamples metadata validator and FAIRsharing registry can help validate metadata. Protocols.io can be used for protocol documentation.</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>For mouse single-cell omics data, deposit in the NIMH Data Archive (NDA) if required by NIMH, or in community repositories such as Gene Expression Omnibus (GEO), ArrayExpress, or Single Cell Expression Atlas. For spatial omics, consider the Brain Image Library (BIL) or the Single Cell Portal (Broad Institute). If data are multi-modal or spatial, ensure the repository supports these formats. Provide persistent identifiers (e.g., accession numbers, DOIs) in publications.</t>
+          <t>De-identification is not required for mouse data, as no human subjects are involved in the initial dataset. If human data are added in the future, follow NIH and NIMH policies: remove all direct and indirect identifiers, and ensure data are shared in accordance with consent and IRB requirements. Update the data sharing plan accordingly.</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>NIH strongly encourages open data sharing. Use the Creative Commons CC0 1.0 Universal (Public Domain Dedication) license for mouse data, as recommended by NIH and major repositories (e.g., GEO, ArrayExpress). If future human data are subject to consent or privacy restrictions, select a license that aligns with those constraints and update documentation accordingly.</t>
+          <t>For mouse data, no de-identification tools are needed. For future human data, use tools such as the NIMH Data Archive (NDA) de-identification guidance, the HIPAA Safe Harbor checklist, and the Open Brain Consent de-identification scripts for omics data.</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>For mouse single-cell omics data, deposit in the Gene Expression Omnibus (GEO) or ArrayExpress for general omics data, and the Single Cell Expression Atlas for single-cell data. For spatial transcriptomics, consider the Brain Image Library (BIL) or the Neuroscience Multi-Omic Archive (NeMO). NIH strongly encourages use of these repositories. If human data are added, use controlled-access repositories such as dbGaP or the NIMH Data Archive (NDA) as appropriate.</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Recommended approach: Use the Creative Commons Attribution 4.0 International (CC BY 4.0) license, which is NIH- and NIMH-compliant and maximizes reuse. If human data are added and consent restricts sharing, use a more restrictive license or controlled-access terms as required by the consent and IRB.</t>
         </is>
       </c>
     </row>
@@ -1032,24 +1115,28 @@
  be uploaded to NDA during the second quarter of the first year of funding. As discussed in the application, 
  structural MRI scans are available for time points before and after treatment along with relevant clinical data.
 Based on these inputs, provide clear, practical, and user-friendly FAIR data guidance organized under the following sections:
-1. Recommended file formats
-Explain which file format(s) should be used for this type of data and why they are appropriate for FAIR sharing and reuse.
-2. Relevant tools and software
-List tools, software, or platforms that can help prepare, convert, validate, organize, document, or share this type of data.
-3. Recommended dataset structure or standard
-State the dataset structure, schema, or community standard that should be followed, if one exists.
-4. Dataset organization details
-Provide detailed guidance on how the dataset should be organized, including folder structure, file naming conventions, table organization, metadata arrangement, versioning considerations, and any other important technical details.
-5. Metadata and documentation files to include
-List the metadata files, README files, data dictionaries, codebooks, protocols, or other documentation that should accompany the dataset.
-6. Tools for metadata preparation and validation
-Suggest tools that can help create, validate, manage, or standardize metadata for this dataset.
-7. De-identification and privacy considerations
-State whether de-identification is required. Explain what should be done based on the subject type, the data modality, and whether the study involves human participants. If consent language affects sharing, explain that clearly.
-8. Recommended repositories
-Suggest appropriate repositories for sharing the data, prioritizing repositories recommended, required, or commonly accepted by the funding source and data type.
-9. Recommended data licenses
-Recommend appropriate data license(s), prioritizing those expected, suggested, or required by the funding source. If restrictions apply because of human subjects or consent limitations, explain that clearly.
+1- Suggested file formats for each data type
+Identify the recommended file format or formats for each data type in the dataset. Briefly explain why these formats are appropriate for FAIR sharing, reuse, interoperability, and long-term preservation.
+2- Tools for converting data to the suggested file formats
+List tools, software, or workflows that can be used to convert raw or source data into the recommended file formats.
+3- Suggested standard structure to organize the dataset
+State the recommended dataset structure, schema, specification, or community standard that should be used to organize the dataset, if one exists.
+4- Tools for organizing the dataset in the suggested structure
+List tools, software, templates, or platforms that can help organize the dataset according to the recommended structure or standard.
+5- Metadata and information that should be provided with the data
+Describe the metadata, documentation, contextual information, data dictionaries, codebooks, README files, protocols, and any other supporting information that should accompany the dataset.
+6- Suggested standard structure and file format for metadata
+State the recommended structure, schema, standard, and file format that should be used for metadata and documentation files included with the dataset.
+7-Tools for preparing metadata in the suggested structure and file format
+List tools, software, validators, templates, or platforms that can help create, manage, standardize, or validate metadata in the recommended structure and format.
+8- Suggested de-identification approach
+State whether de-identification is required. Explain the recommended de-identification or privacy-preserving approach based on the subject type, data modality, sensitivity of the data, and whether human participants are involved. If consent language affects sharing, explain that clearly.
+9- Tools to implement the suggested de-identification approach
+List tools, software, workflows, or methods that can help implement the recommended de-identification or privacy protection approach.
+10-Suggested repositories for sharing the dataset
+Recommend appropriate repositories for sharing the dataset, prioritizing repositories required, recommended, or commonly accepted by the funding source, subject type, and data modality.
+11- Suggested license for sharing the dataset
+Recommend an appropriate data license or licensing approach, prioritizing what is expected, suggested, or required by the funding source. If restrictions apply because of human subjects, controlled access, or consent limitations, explain that clearly.
 Instructions for your response:
 - Make the guidance practical, concise, and easy for researchers to follow.
 - Tailor all recommendations to the combination of funding source, human-subject status, consent language, and data modality.
@@ -1060,76 +1147,96 @@
 Return your answer in valid JSON format only.
 Use exactly this JSON structure:
 {
-  "Recommended file formats": "",
-  "Relevant tools and software": "",
-  "Recommended dataset structure or standard": "",
-  "Dataset organization details": "",
-  "Metadata and documentation files to include": "",
-  "Tools for metadata preparation and validation": "",
-  "De-identification and privacy considerations": "",
-  "Recommended repositories": "",
-  "Recommended data licenses": ""
+  "1-Suggested file formats for each data type": "",
+  "2-Tools for converting data to the suggested file formats": "",
+  "3-Suggested standard structure to organize the dataset": "",
+  "4-Tools for organizing the dataset in the suggested structure": "",
+  "5-Metadata and information that should be provided with the data": "",
+  "6-Suggested standard structure and file format for metadata": "",
+  "7-Tools for preparing metadata in the suggested structure and file format": "",
+  "8-Suggested de-identification approach": "",
+  "9-Tools to implement the suggested de-identification approach": "",
+  "10-Suggested repositories for sharing the dataset": "",
+  "11-Suggested license for sharing the dataset": ""
 }</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>{
-  "Recommended file formats": "For MRI images, use NIfTI (.nii or .nii.gz) format, which is the community standard for neuroimaging and is required by the NIMH Data Archive (NDA). For clinical assessments and tabular data, use non-proprietary, machine-readable formats such as CSV (.csv) or TSV (.tsv). Avoid proprietary formats (e.g., Excel .xls/.xlsx) for primary data files to maximize interoperability and reuse.",
-  "Relevant tools and software": "Use MRI data conversion and validation tools such as dcm2niix (for converting DICOM to NIfTI), BIDS Validator (for checking dataset structure), and MRIcron or FSLeyes (for visual inspection). For organizing and preparing data, use the BIDS Starter Kit and NDA Data Dictionary Tool. For metadata, use the NDA's Data Dictionary and Data Submission tools. For de-identification, use pydeface or mri_deface for MRI images.",
-  "Recommended dataset structure or standard": "Follow the Brain Imaging Data Structure (BIDS) standard for organizing MRI data and associated clinical/behavioral data. BIDS is widely adopted in neuroimaging, required by many repositories, and facilitates interoperability and reuse. For NDA submissions, ensure compliance with NDA's data dictionary and submission requirements, which are compatible with BIDS.",
-  "Dataset organization details": "Organize data in a BIDS-compliant folder structure: a root directory with subfolders for each subject (e.g., sub-001), session (if applicable), and modality (e.g., anat for anatomical MRI). Use standardized BIDS file naming conventions (e.g., sub-001_ses-pre_anat.nii.gz). Store clinical/behavioral data in tabular files (e.g., participants.tsv, clinical_assessments.tsv) with clear column headers. Include a dataset_description.json file at the root. Maintain a README file and a CHANGES log for versioning. For NDA, map variables to the NDA data dictionary and ensure all required metadata fields are completed.",
-  "Metadata and documentation files to include": "Include a README file describing the dataset, a dataset_description.json (per BIDS), a data dictionary/codebook for all tabular data, and protocols for data collection and processing. For NDA, provide the NDA-required data dictionary and data structure documentation. Include a CHANGES file to document updates. If scripts or code are used for preprocessing, include these with documentation.",
-  "Tools for metadata preparation and validation": "Use the BIDS Validator (online or command-line) to check BIDS compliance. Use the NDA Data Dictionary Tool for preparing and validating NDA metadata. For general metadata management, tools like DataLad or OpenNeuro's BIDS tools can assist. For tabular data, use csvlint or similar tools to check formatting.",
-  "De-identification and privacy considerations": "De-identification is required for all shared human subjects data. For MRI images, remove all facial features using tools like pydeface or mri_deface, and strip all personal identifiers from image headers. For clinical data, remove direct identifiers (names, dates of birth, addresses, etc.) and use subject codes. Since all participants are consented for broad data sharing, data can be shared in public repositories, but ensure all de-identification steps are documented and compliant with NIH and NDA policies.",
-  "Recommended repositories": "Deposit all data in the NIMH Data Archive (NDA), which is the NIH-designated repository for mental health research data and required for NIMH-funded studies. For BIDS-compliant neuroimaging data, OpenNeuro is also a widely used repository, but NDA should be prioritized to meet funder requirements. Reference existing NDA collections (2134, 2433) and create a new collection for the newly shared data.",
-  "Recommended data licenses": "Use the NDA Data Use Certification (DUC) and associated data sharing agreements, which govern data access and reuse for human subjects data in NDA. For OpenNeuro or other repositories, use the Creative Commons Attribution 4.0 International (CC BY 4.0) license if permitted by consent and institutional policy. Always ensure the selected license aligns with participant consent for broad data sharing and NIH policy."
+  "1-Suggested file formats for each data type": {
+    "MRI images": "NIfTI (.nii or .nii.gz) is recommended for structural MRI data. NIfTI is an open, widely adopted neuroimaging format that supports interoperability, long-term preservation, and is required by many repositories including the NIMH Data Archive (NDA).",
+    "Clinical assessments": "Tabular data should be provided in CSV (.csv) or TSV (.tsv) format. These are open, non-proprietary formats that are machine-readable, widely supported, and facilitate reuse and interoperability."
+  },
+  "2-Tools for converting data to the suggested file formats": {
+    "MRI images": "dcm2niix is a widely used tool for converting DICOM files to NIfTI format.",
+    "Clinical assessments": "Spreadsheet software (e.g., Microsoft Excel, LibreOffice Calc, Google Sheets) can export data to CSV or TSV. For more complex data, Python (pandas) or R can be used to convert and clean tabular data."
+  },
+  "3-Suggested standard structure to organize the dataset": "The Brain Imaging Data Structure (BIDS) is the recommended community standard for organizing MRI and associated clinical data. BIDS provides a clear folder hierarchy, naming conventions, and metadata requirements to maximize interoperability and reuse.",
+  "4-Tools for organizing the dataset in the suggested structure": "BIDS Starter Kit (templates and guides), BIDScoin (semi-automated conversion), HeuDiConv (DICOM to BIDS conversion), and the BIDS Validator (for checking compliance) are recommended tools for organizing and validating datasets according to BIDS.",
+  "5-Metadata and information that should be provided with the data": "Provide a comprehensive README file describing the dataset, study design, and data collection protocols. Include a data dictionary/codebook for all clinical variables, details of MRI acquisition parameters, preprocessing steps, and any relevant protocols. Participant consent language and IRB approval documentation should be included or referenced. For BIDS, required metadata files include dataset_description.json, participants.tsv, and accompanying JSON sidecars for imaging data.",
+  "6-Suggested standard structure and file format for metadata": "Use the BIDS metadata structure, which includes JSON files for imaging metadata (e.g., dataset_description.json, *_T1w.json), TSV files for participant and session information, and plain text (README, CHANGES). For clinical data, provide a data dictionary in CSV, TSV, or JSON format.",
+  "7-Tools for preparing metadata in the suggested structure and file format": "BIDS Starter Kit (metadata templates), BIDS Validator (checks completeness and correctness), BIDScoin and HeuDiConv (generate metadata during conversion), and spreadsheet editors for TSV/CSV files. NDA also provides data dictionary templates and validation tools for submission.",
+  "8-Suggested de-identification approach": "De-identification is required for all human subject data. For MRI, remove all facial features from images (defacing) and strip DICOM headers of PHI. For clinical data, remove direct identifiers (names, dates of birth, addresses, etc.) and use study-specific participant IDs. Since participants are consented for broad sharing, data can be shared under controlled access with appropriate safeguards.",
+  "9-Tools to implement the suggested de-identification approach": "For MRI: pydeface, mri_deface, or FSL's deface for removing facial features; dcm2niix for removing PHI from headers. For clinical data: Python (pandas), R, or NDA-provided de-identification tools to remove or pseudonymize identifiers.",
+  "10-Suggested repositories for sharing the dataset": "The NIMH Data Archive (NDA) is the required repository for NIMH-funded human subjects data, including MRI and clinical assessments. NDA supports controlled access and is designed for compliance with NIH data sharing policies.",
+  "11-Suggested license for sharing the dataset": "NDA requires data to be shared under a controlled access model, not an open license. Data use is governed by NDA Data Use Certification Agreements, which ensure compliance with participant consent and privacy requirements. Explicitly state in documentation that data are available for secondary use via NDA under controlled access."
 }</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>For MRI images, use NIfTI (.nii or .nii.gz) format, which is the community standard for neuroimaging and is required by the NIMH Data Archive (NDA). For clinical assessments and tabular data, use non-proprietary, machine-readable formats such as CSV (.csv) or TSV (.tsv). Avoid proprietary formats (e.g., Excel .xls/.xlsx) for primary data files to maximize interoperability and reuse.</t>
+          <t>{'MRI images': 'NIfTI (.nii or .nii.gz) is recommended for structural MRI data. NIfTI is an open, widely adopted neuroimaging format that supports interoperability, long-term preservation, and is required by many repositories including the NIMH Data Archive (NDA).', 'Clinical assessments': 'Tabular data should be provided in CSV (.csv) or TSV (.tsv) format. These are open, non-proprietary formats that are machine-readable, widely supported, and facilitate reuse and interoperability.'}</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Use MRI data conversion and validation tools such as dcm2niix (for converting DICOM to NIfTI), BIDS Validator (for checking dataset structure), and MRIcron or FSLeyes (for visual inspection). For organizing and preparing data, use the BIDS Starter Kit and NDA Data Dictionary Tool. For metadata, use the NDA's Data Dictionary and Data Submission tools. For de-identification, use pydeface or mri_deface for MRI images.</t>
+          <t>{'MRI images': 'dcm2niix is a widely used tool for converting DICOM files to NIfTI format.', 'Clinical assessments': 'Spreadsheet software (e.g., Microsoft Excel, LibreOffice Calc, Google Sheets) can export data to CSV or TSV. For more complex data, Python (pandas) or R can be used to convert and clean tabular data.'}</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Follow the Brain Imaging Data Structure (BIDS) standard for organizing MRI data and associated clinical/behavioral data. BIDS is widely adopted in neuroimaging, required by many repositories, and facilitates interoperability and reuse. For NDA submissions, ensure compliance with NDA's data dictionary and submission requirements, which are compatible with BIDS.</t>
+          <t>The Brain Imaging Data Structure (BIDS) is the recommended community standard for organizing MRI and associated clinical data. BIDS provides a clear folder hierarchy, naming conventions, and metadata requirements to maximize interoperability and reuse.</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Organize data in a BIDS-compliant folder structure: a root directory with subfolders for each subject (e.g., sub-001), session (if applicable), and modality (e.g., anat for anatomical MRI). Use standardized BIDS file naming conventions (e.g., sub-001_ses-pre_anat.nii.gz). Store clinical/behavioral data in tabular files (e.g., participants.tsv, clinical_assessments.tsv) with clear column headers. Include a dataset_description.json file at the root. Maintain a README file and a CHANGES log for versioning. For NDA, map variables to the NDA data dictionary and ensure all required metadata fields are completed.</t>
+          <t>BIDS Starter Kit (templates and guides), BIDScoin (semi-automated conversion), HeuDiConv (DICOM to BIDS conversion), and the BIDS Validator (for checking compliance) are recommended tools for organizing and validating datasets according to BIDS.</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Include a README file describing the dataset, a dataset_description.json (per BIDS), a data dictionary/codebook for all tabular data, and protocols for data collection and processing. For NDA, provide the NDA-required data dictionary and data structure documentation. Include a CHANGES file to document updates. If scripts or code are used for preprocessing, include these with documentation.</t>
+          <t>Provide a comprehensive README file describing the dataset, study design, and data collection protocols. Include a data dictionary/codebook for all clinical variables, details of MRI acquisition parameters, preprocessing steps, and any relevant protocols. Participant consent language and IRB approval documentation should be included or referenced. For BIDS, required metadata files include dataset_description.json, participants.tsv, and accompanying JSON sidecars for imaging data.</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Use the BIDS Validator (online or command-line) to check BIDS compliance. Use the NDA Data Dictionary Tool for preparing and validating NDA metadata. For general metadata management, tools like DataLad or OpenNeuro's BIDS tools can assist. For tabular data, use csvlint or similar tools to check formatting.</t>
+          <t>Use the BIDS metadata structure, which includes JSON files for imaging metadata (e.g., dataset_description.json, *_T1w.json), TSV files for participant and session information, and plain text (README, CHANGES). For clinical data, provide a data dictionary in CSV, TSV, or JSON format.</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>De-identification is required for all shared human subjects data. For MRI images, remove all facial features using tools like pydeface or mri_deface, and strip all personal identifiers from image headers. For clinical data, remove direct identifiers (names, dates of birth, addresses, etc.) and use subject codes. Since all participants are consented for broad data sharing, data can be shared in public repositories, but ensure all de-identification steps are documented and compliant with NIH and NDA policies.</t>
+          <t>BIDS Starter Kit (metadata templates), BIDS Validator (checks completeness and correctness), BIDScoin and HeuDiConv (generate metadata during conversion), and spreadsheet editors for TSV/CSV files. NDA also provides data dictionary templates and validation tools for submission.</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Deposit all data in the NIMH Data Archive (NDA), which is the NIH-designated repository for mental health research data and required for NIMH-funded studies. For BIDS-compliant neuroimaging data, OpenNeuro is also a widely used repository, but NDA should be prioritized to meet funder requirements. Reference existing NDA collections (2134, 2433) and create a new collection for the newly shared data.</t>
+          <t>De-identification is required for all human subject data. For MRI, remove all facial features from images (defacing) and strip DICOM headers of PHI. For clinical data, remove direct identifiers (names, dates of birth, addresses, etc.) and use study-specific participant IDs. Since participants are consented for broad sharing, data can be shared under controlled access with appropriate safeguards.</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Use the NDA Data Use Certification (DUC) and associated data sharing agreements, which govern data access and reuse for human subjects data in NDA. For OpenNeuro or other repositories, use the Creative Commons Attribution 4.0 International (CC BY 4.0) license if permitted by consent and institutional policy. Always ensure the selected license aligns with participant consent for broad data sharing and NIH policy.</t>
+          <t>For MRI: pydeface, mri_deface, or FSL's deface for removing facial features; dcm2niix for removing PHI from headers. For clinical data: Python (pandas), R, or NDA-provided de-identification tools to remove or pseudonymize identifiers.</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>The NIMH Data Archive (NDA) is the required repository for NIMH-funded human subjects data, including MRI and clinical assessments. NDA supports controlled access and is designed for compliance with NIH data sharing policies.</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>NDA requires data to be shared under a controlled access model, not an open license. Data use is governed by NDA Data Use Certification Agreements, which ensure compliance with participant consent and privacy requirements. Explicitly state in documentation that data are available for secondary use via NDA under controlled access.</t>
         </is>
       </c>
     </row>

</xml_diff>